<commit_message>
task-2360: calibrate review lane against Excel (search, special, errors, watch fixtures and fixes)
</commit_message>
<xml_diff>
--- a/crates/unluminous-sheet/tests/fixtures/review/search.xlsx
+++ b/crates/unluminous-sheet/tests/fixtures/review/search.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\jason\dev\unluminous\.claude\worktrees\agent-ace8b8f091fdee255\crates\unluminous-sheet\tests\fixtures\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{589A7847-5EBF-4E4C-A601-A7F5511085BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CDE82280-2761-47AF-BEAB-F8FEBCFA1982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1875" yWindow="6660" windowWidth="43200" windowHeight="23445" activeTab="1" xr2:uid="{8270C57E-7000-4E11-81F9-ED74A820D457}"/>
+    <workbookView xWindow="1875" yWindow="6660" windowWidth="43200" windowHeight="23445" activeTab="1" xr2:uid="{D12135A3-DF63-4346-A82F-D55A0736EE88}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,11 +42,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>Probe Author</author>
-    <author>tc={6026C553-43BB-4B45-98B2-A13F65EE8B27}</author>
+    <author>Oracle</author>
+    <author>tc={C4CAC2E1-FBC0-4F31-8563-E91A4D00DC91}</author>
   </authors>
   <commentList>
-    <comment ref="A9" authorId="0" shapeId="0" xr:uid="{5249F423-D3C8-4361-8771-2E7821913B86}">
+    <comment ref="A9" authorId="0" shapeId="0" xr:uid="{83F2C356-6058-435E-A41C-934E1BD92B9B}">
       <text>
         <r>
           <rPr>
@@ -60,7 +60,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B9" authorId="0" shapeId="0" xr:uid="{2C199A02-2383-4E3F-9054-153B5CFCAC6D}">
+    <comment ref="B9" authorId="0" shapeId="0" xr:uid="{3E860515-EAC5-4A0D-BCB9-616C22AB574A}">
       <text>
         <r>
           <rPr>
@@ -74,7 +74,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C9" authorId="1" shapeId="0" xr:uid="{6026C553-43BB-4B45-98B2-A13F65EE8B27}">
+    <comment ref="C9" authorId="1" shapeId="0" xr:uid="{C4CAC2E1-FBC0-4F31-8563-E91A4D00DC91}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -254,7 +254,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Jason McAffee" id="{6049335B-6D45-42BA-BE63-5BE5D54AB81E}" userId="1c91cd66ecc6bf30" providerId="Windows Live"/>
+  <person displayName="Oracle" id="{D4582047-96CD-491C-A9FE-9355757DDA37}" userId="Oracle" providerId="None"/>
 </personList>
 </file>
 
@@ -575,17 +575,17 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C9" dT="2026-10-24T19:53:55.67" personId="{6049335B-6D45-42BA-BE63-5BE5D54AB81E}" id="{6026C553-43BB-4B45-98B2-A13F65EE8B27}">
+  <threadedComment ref="C9" dT="2026-10-25T09:00:22.36" personId="{D4582047-96CD-491C-A9FE-9355757DDA37}" id="{C4CAC2E1-FBC0-4F31-8563-E91A4D00DC91}">
     <text>apple thread</text>
   </threadedComment>
-  <threadedComment ref="C9" dT="2026-10-24T19:53:56.18" personId="{6049335B-6D45-42BA-BE63-5BE5D54AB81E}" id="{3688D651-F724-4E8B-92FB-4312383981F0}" parentId="{6026C553-43BB-4B45-98B2-A13F65EE8B27}">
+  <threadedComment ref="C9" dT="2026-10-25T09:00:22.42" personId="{D4582047-96CD-491C-A9FE-9355757DDA37}" id="{2AC9B0F9-7AB9-4148-AC4F-6DD61E107CB6}" parentId="{C4CAC2E1-FBC0-4F31-8563-E91A4D00DC91}">
     <text>banana reply</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{112929DA-0E0D-4678-9791-D2E7CA1701E4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0ED2244-E73E-454C-ABF4-04198045CC64}">
   <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -723,7 +723,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2C27A52-7FF4-47FF-85B3-38E3D878921A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CFC7DDA-39BB-4D50-9C8B-8DB61C49C4C5}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>